<commit_message>
data: refresh CareerONE jobs (2026-06-18)
</commit_message>
<xml_diff>
--- a/careerone_jobs.xlsx
+++ b/careerone_jobs.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V57"/>
+  <dimension ref="A1:V58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
@@ -7042,6 +7042,96 @@
       </c>
       <c r="V57" t="inlineStr"/>
     </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Finance and Administration officer</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Consultancy / Contract</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr"/>
+      <c r="D58" t="inlineStr"/>
+      <c r="E58" t="inlineStr"/>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>Development / NGO</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr"/>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>– [Your Name]”
+to the following email address:
+[email protected]
+The deadline for applications is
+July 06
+th
+, 2026.
+Additional information:
+Expected start date:
+July 15
+th
+, 2026
+1st selection (document screening) – 2nd selection ((interview, can be skipped depends on the situation) – Final selection (interview).
+Initial contract: 1 year, with the possibility of extension based on performance and project needs.
+The position may be filled before the deadline if a suitable candidate is found.</t>
+        </is>
+      </c>
+      <c r="J58" t="inlineStr">
+        <is>
+          <t>hoaanh.dao@hotmail.com</t>
+        </is>
+      </c>
+      <c r="K58" t="inlineStr">
+        <is>
+          <t>https://en-m.miral.org</t>
+        </is>
+      </c>
+      <c r="L58" t="inlineStr">
+        <is>
+          <t>MWF</t>
+        </is>
+      </c>
+      <c r="M58" t="inlineStr"/>
+      <c r="N58" t="inlineStr">
+        <is>
+          <t>NGO / Development</t>
+        </is>
+      </c>
+      <c r="O58" t="inlineStr"/>
+      <c r="P58" t="inlineStr">
+        <is>
+          <t>NGO / Development</t>
+        </is>
+      </c>
+      <c r="Q58" t="inlineStr">
+        <is>
+          <t>https://en-m.miral.org</t>
+        </is>
+      </c>
+      <c r="R58" t="inlineStr"/>
+      <c r="S58" t="inlineStr"/>
+      <c r="T58" t="inlineStr">
+        <is>
+          <t>https://careerone.vn/jobs/finance-and-administration-officer-2/</t>
+        </is>
+      </c>
+      <c r="U58" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="V58" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>